<commit_message>
`Removed entire CVE search system codebase`
</commit_message>
<xml_diff>
--- a/data/Yash Asset List.xlsx
+++ b/data/Yash Asset List.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{FED7D8E7-E9B1-4B0E-A854-C80FB80D2ED1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{4F7E630A-9C12-404F-8245-177BD3D80BE8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE0A167C-1026-4BD4-973D-65076F5E8EA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2723,21 +2723,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:J177"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="38.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="38.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="40.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="37.799999999999997" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>600</v>
       </c>
@@ -2769,7 +2769,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2865,7 +2865,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3185,7 +3185,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3217,7 +3217,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3249,7 +3249,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3313,7 +3313,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3345,7 +3345,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3441,7 +3441,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3537,7 +3537,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3569,7 +3569,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -3665,7 +3665,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -3729,7 +3729,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -3825,7 +3825,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -3857,7 +3857,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -3921,7 +3921,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -3953,7 +3953,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -3985,7 +3985,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -4017,7 +4017,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -4049,7 +4049,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -4113,7 +4113,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -4145,7 +4145,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -4177,7 +4177,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -4401,7 +4401,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -4433,7 +4433,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -4465,7 +4465,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -4497,7 +4497,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -4561,7 +4561,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -4593,7 +4593,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -4689,7 +4689,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -4721,7 +4721,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -4753,7 +4753,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -4785,7 +4785,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -4817,7 +4817,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -4849,7 +4849,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -4881,7 +4881,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -4913,7 +4913,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -4945,7 +4945,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -5009,7 +5009,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -5073,7 +5073,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -5105,7 +5105,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -5137,7 +5137,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -5169,7 +5169,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -5201,7 +5201,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -5265,7 +5265,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -5329,7 +5329,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -5361,7 +5361,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -5393,7 +5393,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -5425,7 +5425,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -5457,7 +5457,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -5489,7 +5489,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -5521,7 +5521,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -5553,7 +5553,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -5585,7 +5585,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -5617,7 +5617,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -5649,7 +5649,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -5681,7 +5681,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -5713,7 +5713,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -5745,7 +5745,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -5777,7 +5777,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -5809,7 +5809,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -5841,7 +5841,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -5873,7 +5873,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -5905,7 +5905,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -5937,7 +5937,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -6001,7 +6001,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -6033,7 +6033,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -6065,7 +6065,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -6161,7 +6161,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -6193,7 +6193,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -6225,7 +6225,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -6257,7 +6257,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -6289,7 +6289,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -6321,7 +6321,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -6353,7 +6353,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -6385,7 +6385,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -6449,7 +6449,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -6481,7 +6481,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -6513,7 +6513,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>118</v>
       </c>
@@ -6545,7 +6545,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -6609,7 +6609,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -6641,7 +6641,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -6673,7 +6673,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -6705,7 +6705,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -6737,7 +6737,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -6769,7 +6769,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -6801,7 +6801,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -6833,7 +6833,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -6865,7 +6865,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -6897,7 +6897,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -6929,7 +6929,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>131</v>
       </c>
@@ -6961,7 +6961,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>132</v>
       </c>
@@ -6993,7 +6993,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>133</v>
       </c>
@@ -7025,7 +7025,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>134</v>
       </c>
@@ -7057,7 +7057,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>135</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="2">
         <v>136</v>
       </c>
@@ -7121,7 +7121,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -7153,7 +7153,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>138</v>
       </c>
@@ -7185,7 +7185,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>139</v>
       </c>
@@ -7217,7 +7217,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>140</v>
       </c>
@@ -7249,7 +7249,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -7281,7 +7281,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>142</v>
       </c>
@@ -7313,7 +7313,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>143</v>
       </c>
@@ -7345,7 +7345,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145" s="2">
         <v>144</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146" s="2">
         <v>145</v>
       </c>
@@ -7409,7 +7409,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="147" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2">
         <v>146</v>
       </c>
@@ -7441,7 +7441,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="148" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -7473,7 +7473,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="149" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>148</v>
       </c>
@@ -7505,7 +7505,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2">
         <v>149</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="151" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>150</v>
       </c>
@@ -7569,7 +7569,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="152" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>151</v>
       </c>
@@ -7601,7 +7601,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="153" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -7633,7 +7633,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="154" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="155" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -7697,7 +7697,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2">
         <v>155</v>
       </c>
@@ -7729,7 +7729,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -7761,7 +7761,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="158" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -7793,7 +7793,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="159" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -7825,7 +7825,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="160" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>159</v>
       </c>
@@ -7857,7 +7857,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="161" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -7889,7 +7889,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="162" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2">
         <v>161</v>
       </c>
@@ -7921,7 +7921,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="163" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -7953,7 +7953,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164" s="2">
         <v>163</v>
       </c>
@@ -7985,7 +7985,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165" s="2">
         <v>164</v>
       </c>
@@ -8015,7 +8015,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>166</v>
       </c>
@@ -8047,7 +8047,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167" s="2">
         <v>167</v>
       </c>
@@ -8077,7 +8077,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168" s="2">
         <v>168</v>
       </c>
@@ -8109,7 +8109,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169" s="2">
         <v>169</v>
       </c>
@@ -8139,7 +8139,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A170" s="2">
         <v>170</v>
       </c>
@@ -8171,7 +8171,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>171</v>
       </c>
@@ -8201,7 +8201,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>172</v>
       </c>
@@ -8233,7 +8233,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A173" s="2">
         <v>173</v>
       </c>
@@ -8263,7 +8263,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A174" s="2">
         <v>174</v>
       </c>
@@ -8295,7 +8295,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A175" s="2">
         <v>175</v>
       </c>
@@ -8325,7 +8325,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A176" s="2">
         <v>176</v>
       </c>
@@ -8357,7 +8357,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A177" s="2">
         <v>177</v>
       </c>
@@ -8434,15 +8434,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EFD2FCB-3583-465F-A9D8-A91024330A02}">
   <dimension ref="A1:G141"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.90625" customWidth="1"/>
-    <col min="7" max="7" width="24.90625" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.88671875" customWidth="1"/>
+    <col min="7" max="7" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
         <v>605</v>
       </c>
@@ -8459,7 +8459,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>10</v>
       </c>
@@ -8474,7 +8474,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
         <v>19</v>
       </c>
@@ -8489,7 +8489,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
         <v>77</v>
       </c>
@@ -8504,7 +8504,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
         <v>83</v>
       </c>
@@ -8519,7 +8519,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
         <v>86</v>
       </c>
@@ -8534,7 +8534,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
         <v>135</v>
       </c>
@@ -8549,7 +8549,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
         <v>168</v>
       </c>
@@ -8564,7 +8564,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="s">
         <v>173</v>
       </c>
@@ -8579,7 +8579,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
         <v>176</v>
       </c>
@@ -8594,7 +8594,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
         <v>209</v>
       </c>
@@ -8609,7 +8609,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="18" t="s">
         <v>269</v>
       </c>
@@ -8624,7 +8624,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
         <v>272</v>
       </c>
@@ -8639,7 +8639,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
         <v>277</v>
       </c>
@@ -8654,7 +8654,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="18" t="s">
         <v>342</v>
       </c>
@@ -8669,7 +8669,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="21" t="s">
         <v>377</v>
       </c>
@@ -8684,7 +8684,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="21" t="s">
         <v>396</v>
       </c>
@@ -8699,7 +8699,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="18" t="s">
         <v>400</v>
       </c>
@@ -8714,7 +8714,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="18" t="s">
         <v>453</v>
       </c>
@@ -8729,7 +8729,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
         <v>457</v>
       </c>
@@ -8744,7 +8744,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="18" t="s">
         <v>466</v>
       </c>
@@ -8759,7 +8759,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="23" t="s">
         <v>490</v>
       </c>
@@ -8774,7 +8774,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="18" t="s">
         <v>493</v>
       </c>
@@ -8789,7 +8789,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="23" t="s">
         <v>549</v>
       </c>
@@ -8804,7 +8804,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
         <v>556</v>
       </c>
@@ -8819,7 +8819,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="23" t="s">
         <v>560</v>
       </c>
@@ -8834,7 +8834,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="23" t="s">
         <v>564</v>
       </c>
@@ -8849,7 +8849,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="23" t="s">
         <v>567</v>
       </c>
@@ -8864,7 +8864,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="23" t="s">
         <v>571</v>
       </c>
@@ -8879,7 +8879,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="23" t="s">
         <v>574</v>
       </c>
@@ -8894,7 +8894,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
         <v>577</v>
       </c>
@@ -8909,7 +8909,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="23" t="s">
         <v>580</v>
       </c>
@@ -8924,7 +8924,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="23" t="s">
         <v>583</v>
       </c>
@@ -8939,7 +8939,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="23" t="s">
         <v>586</v>
       </c>
@@ -8954,7 +8954,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="23" t="s">
         <v>590</v>
       </c>
@@ -8967,7 +8967,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="23" t="s">
         <v>593</v>
       </c>
@@ -8980,7 +8980,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="23" t="s">
         <v>598</v>
       </c>
@@ -8993,7 +8993,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C38" s="3"/>
       <c r="E38" s="3" t="s">
         <v>182</v>
@@ -9002,7 +9002,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C39" s="3"/>
       <c r="E39" s="3" t="s">
         <v>185</v>
@@ -9011,7 +9011,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C40" s="3"/>
       <c r="E40" s="3" t="s">
         <v>188</v>
@@ -9020,7 +9020,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C41" s="3"/>
       <c r="E41" s="3" t="s">
         <v>191</v>
@@ -9029,7 +9029,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C42" s="3"/>
       <c r="E42" s="3" t="s">
         <v>194</v>
@@ -9038,7 +9038,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C43" s="3"/>
       <c r="E43" s="3" t="s">
         <v>197</v>
@@ -9047,7 +9047,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C44" s="3"/>
       <c r="E44" s="3" t="s">
         <v>200</v>
@@ -9056,7 +9056,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C45" s="3"/>
       <c r="E45" s="3" t="s">
         <v>203</v>
@@ -9065,7 +9065,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C46" s="3"/>
       <c r="E46" s="3" t="s">
         <v>206</v>
@@ -9074,7 +9074,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C47" s="3"/>
       <c r="E47" s="3" t="s">
         <v>214</v>
@@ -9083,7 +9083,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C48" s="3"/>
       <c r="E48" s="3" t="s">
         <v>217</v>
@@ -9092,7 +9092,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C49" s="3"/>
       <c r="E49" s="3" t="s">
         <v>220</v>
@@ -9101,7 +9101,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C50" s="3"/>
       <c r="E50" s="3" t="s">
         <v>223</v>
@@ -9110,7 +9110,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C51" s="3"/>
       <c r="E51" s="3" t="s">
         <v>226</v>
@@ -9119,7 +9119,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C52" s="3"/>
       <c r="E52" s="3" t="s">
         <v>229</v>
@@ -9128,7 +9128,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C53" s="3"/>
       <c r="E53" s="3" t="s">
         <v>232</v>
@@ -9137,7 +9137,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C54" s="3"/>
       <c r="E54" s="3" t="s">
         <v>235</v>
@@ -9146,7 +9146,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C55" s="3"/>
       <c r="E55" s="3" t="s">
         <v>238</v>
@@ -9155,7 +9155,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C56" s="3"/>
       <c r="E56" s="3" t="s">
         <v>241</v>
@@ -9164,7 +9164,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C57" s="3"/>
       <c r="E57" s="3" t="s">
         <v>244</v>
@@ -9173,7 +9173,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C58" s="3"/>
       <c r="E58" s="3" t="s">
         <v>247</v>
@@ -9182,7 +9182,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C59" s="3"/>
       <c r="E59" s="3" t="s">
         <v>250</v>
@@ -9191,7 +9191,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C60" s="3"/>
       <c r="E60" s="3" t="s">
         <v>253</v>
@@ -9200,7 +9200,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C61" s="3"/>
       <c r="E61" s="3" t="s">
         <v>257</v>
@@ -9209,7 +9209,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C62" s="3"/>
       <c r="E62" s="3" t="s">
         <v>260</v>
@@ -9218,7 +9218,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C63" s="3"/>
       <c r="E63" s="3" t="s">
         <v>263</v>
@@ -9227,7 +9227,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C64" s="3"/>
       <c r="E64" s="3" t="s">
         <v>266</v>
@@ -9236,7 +9236,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C65" s="3"/>
       <c r="E65" s="3" t="s">
         <v>282</v>
@@ -9245,7 +9245,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="66" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C66" s="3"/>
       <c r="E66" s="3" t="s">
         <v>285</v>
@@ -9254,7 +9254,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C67" s="3"/>
       <c r="E67" s="3" t="s">
         <v>288</v>
@@ -9263,7 +9263,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="68" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C68" s="3"/>
       <c r="E68" s="3" t="s">
         <v>291</v>
@@ -9272,7 +9272,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C69" s="3"/>
       <c r="E69" s="3" t="s">
         <v>294</v>
@@ -9281,7 +9281,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C70" s="3"/>
       <c r="E70" s="3" t="s">
         <v>297</v>
@@ -9290,7 +9290,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="71" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C71" s="14"/>
       <c r="E71" s="3" t="s">
         <v>300</v>
@@ -9299,7 +9299,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="72" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C72" s="3"/>
       <c r="E72" s="14" t="s">
         <v>303</v>
@@ -9308,7 +9308,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="73" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C73" s="3"/>
       <c r="E73" s="3" t="s">
         <v>306</v>
@@ -9317,7 +9317,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C74" s="3"/>
       <c r="E74" s="3" t="s">
         <v>309</v>
@@ -9326,7 +9326,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="75" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="75" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C75" s="3"/>
       <c r="E75" s="3" t="s">
         <v>312</v>
@@ -9335,7 +9335,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C76" s="3"/>
       <c r="E76" s="3" t="s">
         <v>315</v>
@@ -9344,7 +9344,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="77" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C77" s="3"/>
       <c r="E77" s="3" t="s">
         <v>318</v>
@@ -9353,7 +9353,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="78" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C78" s="3"/>
       <c r="E78" s="3" t="s">
         <v>321</v>
@@ -9362,7 +9362,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="79" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C79" s="3"/>
       <c r="E79" s="3" t="s">
         <v>324</v>
@@ -9371,7 +9371,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="80" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C80" s="3"/>
       <c r="E80" s="3" t="s">
         <v>327</v>
@@ -9380,7 +9380,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="81" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="81" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C81" s="3"/>
       <c r="E81" s="3" t="s">
         <v>330</v>
@@ -9389,7 +9389,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="82" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C82" s="3"/>
       <c r="E82" s="3" t="s">
         <v>333</v>
@@ -9398,7 +9398,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="83" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C83" s="3"/>
       <c r="E83" s="3" t="s">
         <v>336</v>
@@ -9407,7 +9407,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="84" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="84" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C84" s="3"/>
       <c r="E84" s="3" t="s">
         <v>339</v>
@@ -9416,7 +9416,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="85" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C85" s="3"/>
       <c r="E85" s="3" t="s">
         <v>347</v>
@@ -9425,7 +9425,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C86" s="3"/>
       <c r="E86" s="3" t="s">
         <v>350</v>
@@ -9434,7 +9434,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="87" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C87" s="3"/>
       <c r="E87" s="3" t="s">
         <v>353</v>
@@ -9443,7 +9443,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="88" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="88" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C88" s="3"/>
       <c r="E88" s="3" t="s">
         <v>356</v>
@@ -9452,7 +9452,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C89" s="14"/>
       <c r="E89" s="3" t="s">
         <v>359</v>
@@ -9461,7 +9461,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="90" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C90" s="3"/>
       <c r="E90" s="14" t="s">
         <v>362</v>
@@ -9470,7 +9470,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="91" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C91" s="3"/>
       <c r="E91" s="3" t="s">
         <v>365</v>
@@ -9479,7 +9479,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="92" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C92" s="14"/>
       <c r="E92" s="3" t="s">
         <v>368</v>
@@ -9488,7 +9488,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="93" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="93" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C93" s="3"/>
       <c r="E93" s="14" t="s">
         <v>371</v>
@@ -9497,7 +9497,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="94" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C94" s="2"/>
       <c r="E94" s="3" t="s">
         <v>374</v>
@@ -9506,7 +9506,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="95" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C95" s="14"/>
       <c r="E95" s="2" t="s">
         <v>381</v>
@@ -9515,7 +9515,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="96" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="96" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C96" s="14"/>
       <c r="E96" s="14" t="s">
         <v>384</v>
@@ -9524,7 +9524,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="97" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C97" s="14"/>
       <c r="E97" s="14" t="s">
         <v>387</v>
@@ -9533,7 +9533,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="98" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C98" s="2"/>
       <c r="E98" s="14" t="s">
         <v>390</v>
@@ -9542,7 +9542,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="99" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C99" s="14"/>
       <c r="E99" s="2" t="s">
         <v>393</v>
@@ -9551,7 +9551,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="100" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="100" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C100" s="3"/>
       <c r="E100" s="14" t="s">
         <v>403</v>
@@ -9560,7 +9560,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="101" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="101" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C101" s="14"/>
       <c r="E101" s="3" t="s">
         <v>406</v>
@@ -9569,7 +9569,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="102" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C102" s="14"/>
       <c r="E102" s="14" t="s">
         <v>409</v>
@@ -9578,7 +9578,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="103" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C103" s="3"/>
       <c r="E103" s="14" t="s">
         <v>412</v>
@@ -9587,7 +9587,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="104" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C104" s="3"/>
       <c r="E104" s="3" t="s">
         <v>415</v>
@@ -9596,7 +9596,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="105" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C105" s="3"/>
       <c r="E105" s="3" t="s">
         <v>418</v>
@@ -9605,7 +9605,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="106" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C106" s="3"/>
       <c r="E106" s="3" t="s">
         <v>423</v>
@@ -9614,7 +9614,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="107" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C107" s="3"/>
       <c r="E107" s="3" t="s">
         <v>426</v>
@@ -9623,7 +9623,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="108" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C108" s="3"/>
       <c r="E108" s="3" t="s">
         <v>429</v>
@@ -9632,7 +9632,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="109" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C109" s="14"/>
       <c r="E109" s="3" t="s">
         <v>432</v>
@@ -9641,7 +9641,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="110" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C110" s="14"/>
       <c r="E110" s="14" t="s">
         <v>435</v>
@@ -9650,7 +9650,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="111" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C111" s="14"/>
       <c r="E111" s="14" t="s">
         <v>438</v>
@@ -9659,7 +9659,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="112" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C112" s="14"/>
       <c r="E112" s="14" t="s">
         <v>441</v>
@@ -9668,7 +9668,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="113" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="113" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C113" s="14"/>
       <c r="E113" s="14" t="s">
         <v>444</v>
@@ -9677,7 +9677,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="114" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="114" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C114" s="14"/>
       <c r="E114" s="14" t="s">
         <v>447</v>
@@ -9686,7 +9686,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="115" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="115" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C115" s="3"/>
       <c r="E115" s="14" t="s">
         <v>450</v>
@@ -9695,7 +9695,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="116" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="116" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C116" s="3"/>
       <c r="E116" s="3" t="s">
         <v>460</v>
@@ -9704,7 +9704,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="117" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="117" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C117" s="3"/>
       <c r="E117" s="3" t="s">
         <v>463</v>
@@ -9713,7 +9713,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="118" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="118" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C118" s="3"/>
       <c r="E118" s="3" t="s">
         <v>469</v>
@@ -9722,7 +9722,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="119" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="119" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C119" s="3"/>
       <c r="E119" s="3" t="s">
         <v>472</v>
@@ -9731,7 +9731,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="120" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="120" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C120" s="3"/>
       <c r="E120" s="3" t="s">
         <v>475</v>
@@ -9740,7 +9740,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="121" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="121" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C121" s="3"/>
       <c r="E121" s="3" t="s">
         <v>478</v>
@@ -9749,7 +9749,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="122" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="122" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C122" s="3"/>
       <c r="E122" s="3" t="s">
         <v>481</v>
@@ -9758,7 +9758,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="123" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="123" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C123" s="3"/>
       <c r="E123" s="3" t="s">
         <v>484</v>
@@ -9767,7 +9767,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="124" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="124" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C124" s="3"/>
       <c r="E124" s="3" t="s">
         <v>487</v>
@@ -9776,7 +9776,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="125" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="125" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C125" s="3"/>
       <c r="E125" s="3" t="s">
         <v>496</v>
@@ -9785,7 +9785,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="126" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="126" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C126" s="3"/>
       <c r="E126" s="3" t="s">
         <v>499</v>
@@ -9794,7 +9794,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="127" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="127" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C127" s="3"/>
       <c r="E127" s="3" t="s">
         <v>502</v>
@@ -9803,7 +9803,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="128" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="128" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C128" s="14"/>
       <c r="E128" s="3" t="s">
         <v>505</v>
@@ -9812,7 +9812,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="129" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C129" s="3"/>
       <c r="E129" s="14" t="s">
         <v>510</v>
@@ -9821,73 +9821,73 @@
         <v>381</v>
       </c>
     </row>
-    <row r="130" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C130" s="3"/>
       <c r="E130" s="3" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="131" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C131" s="3"/>
       <c r="E131" s="3" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="132" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C132" s="3"/>
       <c r="E132" s="3" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="133" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C133" s="3"/>
       <c r="E133" s="3" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="134" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C134" s="3"/>
       <c r="E134" s="3" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="135" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C135" s="3"/>
       <c r="E135" s="3" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="136" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C136" s="3"/>
       <c r="E136" s="3" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="137" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="137" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C137" s="3"/>
       <c r="E137" s="3" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="138" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="138" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C138" s="3"/>
       <c r="E138" s="3" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="139" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="139" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C139" s="3"/>
       <c r="E139" s="3" t="s">
         <v>540</v>
       </c>
     </row>
-    <row r="140" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="140" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C140" s="3"/>
       <c r="E140" s="3" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="141" spans="3:7" x14ac:dyDescent="0.35">
+    <row r="141" spans="3:7" x14ac:dyDescent="0.3">
       <c r="E141" s="3" t="s">
         <v>546</v>
       </c>
@@ -9980,14 +9980,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="278681c7-35fd-409b-af5b-92ccc9bed3f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008085E0EFD0909842AC370FEE43C297B3" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="21f70726adf691c36d64e4206a3ca412">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d" xmlns:ns4="278681c7-35fd-409b-af5b-92ccc9bed3f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3112f7d685964fb1551dbda076e7439a" ns3:_="" ns4:_="">
     <xsd:import namespace="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d"/>
@@ -10240,6 +10232,14 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="278681c7-35fd-409b-af5b-92ccc9bed3f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7AB91C0-F685-4F3B-A8DE-F857E012BABC}">
   <ds:schemaRefs>
@@ -10249,23 +10249,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE9AE2C9-DE78-4CDB-9CC0-1F8211E728DB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="278681c7-35fd-409b-af5b-92ccc9bed3f6"/>
-    <ds:schemaRef ds:uri="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEDDC3D4-FFA0-4E7F-8888-A9F793BF8B4B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10282,4 +10265,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE9AE2C9-DE78-4CDB-9CC0-1F8211E728DB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="278681c7-35fd-409b-af5b-92ccc9bed3f6"/>
+    <ds:schemaRef ds:uri="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
`Updated report.py and export_excel.py to use "Asset IPV4" instead of "Asset Name" in various places.`
</commit_message>
<xml_diff>
--- a/data/Yash Asset List.xlsx
+++ b/data/Yash Asset List.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE0A167C-1026-4BD4-973D-65076F5E8EA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82ADFCFB-6277-4F46-A164-16BC9A4F2A28}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2721,7 +2721,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:J177"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2833,7 +2832,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2865,7 +2864,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2897,7 +2896,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2929,7 +2928,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2961,7 +2960,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2993,7 +2992,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -3025,7 +3024,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -3057,7 +3056,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -3089,7 +3088,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -3121,7 +3120,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -3153,7 +3152,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -3185,7 +3184,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -3217,7 +3216,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3249,7 +3248,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3281,7 +3280,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3409,7 +3408,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3441,7 +3440,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -3473,7 +3472,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -3505,7 +3504,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -3537,7 +3536,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -3569,7 +3568,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -3601,7 +3600,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -3633,7 +3632,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -3665,7 +3664,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -3697,7 +3696,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -3729,7 +3728,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -3761,7 +3760,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -3793,7 +3792,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -3825,7 +3824,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -3889,7 +3888,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -3921,7 +3920,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -3953,7 +3952,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -3985,7 +3984,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -4017,7 +4016,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -4049,7 +4048,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -4081,7 +4080,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -4209,7 +4208,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -4241,7 +4240,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -4273,7 +4272,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -4305,7 +4304,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -4337,7 +4336,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -4369,7 +4368,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -4401,7 +4400,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -4433,7 +4432,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -4465,7 +4464,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -4529,7 +4528,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -4561,7 +4560,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -4593,7 +4592,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -4625,7 +4624,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -4657,7 +4656,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -4689,7 +4688,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -4721,7 +4720,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -4753,7 +4752,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -4785,7 +4784,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -4817,7 +4816,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -4849,7 +4848,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -4881,7 +4880,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -4913,7 +4912,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -4945,7 +4944,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -4977,7 +4976,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -5009,7 +5008,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -5041,7 +5040,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -5073,7 +5072,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -5201,7 +5200,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -5233,7 +5232,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -5265,7 +5264,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -5297,7 +5296,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -5329,7 +5328,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -5361,7 +5360,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -5393,7 +5392,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -5425,7 +5424,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -5457,7 +5456,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -5489,7 +5488,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -5521,7 +5520,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -5553,7 +5552,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -5585,7 +5584,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -5617,7 +5616,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -5649,7 +5648,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="92" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -5681,7 +5680,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -5713,7 +5712,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -5745,7 +5744,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -5777,7 +5776,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="96" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -5809,7 +5808,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="97" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -5873,7 +5872,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -5905,7 +5904,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="100" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -5937,7 +5936,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -5969,7 +5968,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -6001,7 +6000,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="103" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -6033,7 +6032,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -6065,7 +6064,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -6097,7 +6096,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -6129,7 +6128,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -6161,7 +6160,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -6225,7 +6224,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -6257,7 +6256,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -6289,7 +6288,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -6321,7 +6320,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -6353,7 +6352,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -6449,7 +6448,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -6481,7 +6480,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -6513,7 +6512,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>118</v>
       </c>
@@ -6545,7 +6544,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -6577,7 +6576,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -6609,7 +6608,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -6641,7 +6640,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -6673,7 +6672,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -6705,7 +6704,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -6737,7 +6736,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -6769,7 +6768,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -6801,7 +6800,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -6833,7 +6832,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -6865,7 +6864,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -6897,7 +6896,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -6929,7 +6928,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>131</v>
       </c>
@@ -7025,7 +7024,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>134</v>
       </c>
@@ -7057,7 +7056,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>135</v>
       </c>
@@ -7121,7 +7120,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -7153,7 +7152,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>138</v>
       </c>
@@ -7185,7 +7184,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>139</v>
       </c>
@@ -7217,7 +7216,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>140</v>
       </c>
@@ -7249,7 +7248,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -7281,7 +7280,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>142</v>
       </c>
@@ -7313,7 +7312,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>143</v>
       </c>
@@ -7409,7 +7408,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="147" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147" s="2">
         <v>146</v>
       </c>
@@ -7441,7 +7440,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="148" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -7473,7 +7472,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="149" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>148</v>
       </c>
@@ -7505,7 +7504,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A150" s="2">
         <v>149</v>
       </c>
@@ -7537,7 +7536,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="151" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>150</v>
       </c>
@@ -7569,7 +7568,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="152" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>151</v>
       </c>
@@ -7601,7 +7600,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="153" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -7633,7 +7632,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="154" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -7665,7 +7664,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="155" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155" s="2">
         <v>154</v>
       </c>
@@ -7697,7 +7696,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A156" s="2">
         <v>155</v>
       </c>
@@ -7729,7 +7728,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>156</v>
       </c>
@@ -7761,7 +7760,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="158" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -7793,7 +7792,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="159" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A159" s="2">
         <v>158</v>
       </c>
@@ -7825,7 +7824,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="160" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>159</v>
       </c>
@@ -7857,7 +7856,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="161" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
         <v>160</v>
       </c>
@@ -7889,7 +7888,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="162" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162" s="2">
         <v>161</v>
       </c>
@@ -7921,7 +7920,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="163" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>162</v>
       </c>
@@ -8388,13 +8387,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J177" xr:uid="{97E3DF32-8FA1-455D-B5B5-371ED3F6B013}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="Critical"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:J177" xr:uid="{97E3DF32-8FA1-455D-B5B5-371ED3F6B013}"/>
   <mergeCells count="7">
     <mergeCell ref="E176:E177"/>
     <mergeCell ref="E164:E165"/>
@@ -9980,6 +9973,14 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="278681c7-35fd-409b-af5b-92ccc9bed3f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008085E0EFD0909842AC370FEE43C297B3" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="21f70726adf691c36d64e4206a3ca412">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d" xmlns:ns4="278681c7-35fd-409b-af5b-92ccc9bed3f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3112f7d685964fb1551dbda076e7439a" ns3:_="" ns4:_="">
     <xsd:import namespace="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d"/>
@@ -10232,14 +10233,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="278681c7-35fd-409b-af5b-92ccc9bed3f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7AB91C0-F685-4F3B-A8DE-F857E012BABC}">
   <ds:schemaRefs>
@@ -10249,6 +10242,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE9AE2C9-DE78-4CDB-9CC0-1F8211E728DB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="278681c7-35fd-409b-af5b-92ccc9bed3f6"/>
+    <ds:schemaRef ds:uri="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEDDC3D4-FFA0-4E7F-8888-A9F793BF8B4B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10265,21 +10275,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE9AE2C9-DE78-4CDB-9CC0-1F8211E728DB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="278681c7-35fd-409b-af5b-92ccc9bed3f6"/>
-    <ds:schemaRef ds:uri="5b5c9810-cf0f-49f5-a7d2-c11fd73f9b4d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>